<commit_message>
Initial version of the final presentation with the textual content and some pictures
</commit_message>
<xml_diff>
--- a/ToDoList.xlsx
+++ b/ToDoList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sloyn\OneDrive\Документы\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dariashushkova/Downloads/studies/computer_science/Prototyping/Autonomous_vehicle_prototype/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EE215B0-D30A-4942-A7D3-D04E98A38AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAEAB64-5CC8-A44C-872F-63A8A0C9797D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="74">
   <si>
     <t>Daria Shushkova</t>
   </si>
@@ -193,13 +193,74 @@
   </si>
   <si>
     <t>Documenting: Measurement protocol of Ir,Ultrasonic Sensors and motor controller. Logging outputs of tested components, wiring manangment, connecting components, main code adjusting after testing (01.06.25)</t>
+  </si>
+  <si>
+    <t>Done 08.06.25</t>
+  </si>
+  <si>
+    <t>For obstacle avoidance sub-states: Refined system-level state machine into timed automata using UPPAAL. Added guards and invariants to model timing constraints. Verified system reactions (sensor checks, motor updates, etc.) against implementation logic. Simulated the model in UPPAAL. Exported and committed the UPPAAL XML model to Git for version tracking.</t>
+  </si>
+  <si>
+    <t>Done 07.06.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For upper-level states: refined system-level state machine into timed automata using UPPAAL. Added guards and invariants to model timing constraints. Verified system reactions (sensor checks, motor updates, etc.) against implementation logic. Simulated the model in UPPAAL. Exported and committed the UPPAAL XML model to Git for version tracking. Finalizing overall UPPAAL model after obstacle avoidannce implementation.
+</t>
+  </si>
+  <si>
+    <t>task8</t>
+  </si>
+  <si>
+    <t>Testing the system (working on unit tests, testing state machine, motor configuration, sensors reactions) (13.06.25)</t>
+  </si>
+  <si>
+    <t>Done 13.06.25</t>
+  </si>
+  <si>
+    <t>task9</t>
+  </si>
+  <si>
+    <t>Testing the system (working on unit tests, testing state machine, motor configuration, sensors reactions) (16.06.25)</t>
+  </si>
+  <si>
+    <t>Testing the system (working on unit tests, testing state machine, motor configuration, sensors reactions, documenting sensors output in log file and upload it to Git) (13.06.25)</t>
+  </si>
+  <si>
+    <t>Testing the system (working on unit tests, testing state machine, motor configuration, sensors reactions, upload the latest working result to Git) (13.06.25)</t>
+  </si>
+  <si>
+    <t>Testing the system (working on unit tests, testing state machine, motor configuration, sensors reactions, upload the latest working result to Git) (16.06.25)</t>
+  </si>
+  <si>
+    <t>Done 16.06.25</t>
+  </si>
+  <si>
+    <t>Testing the system (working on unit tests, testing state machine, motor configuration, sensors reactions) (20.06.25)</t>
+  </si>
+  <si>
+    <t>Done 20.06.25</t>
+  </si>
+  <si>
+    <t>Testing the system (working on unit tests, testing state machine, motor configuration, sensors reactions, upload the latest working result to Git) (20.06.25)</t>
+  </si>
+  <si>
+    <t>task10</t>
+  </si>
+  <si>
+    <t>task11</t>
+  </si>
+  <si>
+    <t>Creating final presentation (22.06.25)</t>
+  </si>
+  <si>
+    <t>Working on the contentent of final presentation (22.06.25)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,6 +281,13 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -243,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -261,26 +329,44 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -553,23 +639,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" customWidth="1"/>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" customWidth="1"/>
-    <col min="4" max="4" width="53.77734375" customWidth="1"/>
-    <col min="5" max="5" width="30.109375" customWidth="1"/>
-    <col min="6" max="6" width="38.109375" customWidth="1"/>
+    <col min="3" max="3" width="30.1640625" customWidth="1"/>
+    <col min="4" max="4" width="53.83203125" customWidth="1"/>
+    <col min="5" max="5" width="30.1640625" customWidth="1"/>
+    <col min="6" max="6" width="38.1640625" customWidth="1"/>
     <col min="7" max="7" width="36.33203125" customWidth="1"/>
-    <col min="8" max="8" width="41.109375" customWidth="1"/>
+    <col min="8" max="8" width="41.1640625" customWidth="1"/>
     <col min="9" max="9" width="22.6640625" customWidth="1"/>
     <col min="10" max="10" width="41.6640625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="28.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="28.1640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
@@ -583,7 +669,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -618,7 +704,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="36.450000000000003" customHeight="1">
+    <row r="3" spans="1:11" ht="36.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -653,7 +739,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="57.45" customHeight="1">
+    <row r="4" spans="1:11" ht="57.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -688,7 +774,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="99" customHeight="1">
+    <row r="5" spans="1:11" ht="99" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -723,7 +809,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="85.8" customHeight="1">
+    <row r="6" spans="1:11" ht="85.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -736,7 +822,7 @@
       <c r="D6" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="7" t="s">
         <v>52</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -758,14 +844,14 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="73.2" customHeight="1">
+    <row r="7" spans="1:11" ht="73.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>42</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -786,79 +872,262 @@
       <c r="I7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="K7" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="127.2" customHeight="1">
-      <c r="A8" s="1">
+    <row r="8" spans="1:11" ht="127.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>56</v>
+      </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
+    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="10">
+        <v>7</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+    </row>
+    <row r="11" spans="1:11" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="10">
+        <v>8</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="10"/>
+    </row>
+    <row r="14" spans="1:11" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="10"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="10">
+        <v>9</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="10"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="10">
+        <v>10</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="11"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="11"/>
+    </row>
+    <row r="20" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="34">
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="K12:K14"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="H12:H14"/>
+    <mergeCell ref="J12:J14"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="I12:I14"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="C9:C11"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="E9:E11"/>
     <mergeCell ref="K9:K11"/>
     <mergeCell ref="F9:F11"/>
     <mergeCell ref="G9:G11"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="J9:J11"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="C9:C11"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="E9:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>